<commit_message>
BMS schematic almost done + components are assigned their footpritns except connectors
</commit_message>
<xml_diff>
--- a/elec/power/Cubesat Power Budget.xlsx
+++ b/elec/power/Cubesat Power Budget.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\BMS\elec\power\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13982774-ADC9-458E-861B-9854E232494A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB026F42-160A-4756-A3DB-2321ADE1B7BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="62">
   <si>
     <t>Subsystem</t>
   </si>
@@ -68,9 +68,6 @@
     <t>Phase Current (mA)</t>
   </si>
   <si>
-    <t>DIssipated Power (mW)</t>
-  </si>
-  <si>
     <t>Phase Resistant (Ω)</t>
   </si>
   <si>
@@ -119,23 +116,116 @@
     <t>UV LCD Board</t>
   </si>
   <si>
-    <t>3x3 LEDs</t>
-  </si>
-  <si>
-    <t>15V</t>
-  </si>
-  <si>
     <t>Number of Cells:</t>
   </si>
   <si>
     <t>Cell Min Voltage:</t>
+  </si>
+  <si>
+    <t>Note</t>
+  </si>
+  <si>
+    <t>UV LCD Board  Total</t>
+  </si>
+  <si>
+    <t>https://www.ti.com/lit/ds/symlink/tlc5940.pdf</t>
+  </si>
+  <si>
+    <t>Dissipated Power (mW)</t>
+  </si>
+  <si>
+    <t>LED Drivers &amp; LEDS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Estimated current drawn for 2*16 LEDs </t>
+  </si>
+  <si>
+    <t>add some redundency</t>
+  </si>
+  <si>
+    <t>8A</t>
+  </si>
+  <si>
+    <t>GNSS</t>
+  </si>
+  <si>
+    <t>SAM-M10Q</t>
+  </si>
+  <si>
+    <t>This is not accounting for dimming the LEDS</t>
+  </si>
+  <si>
+    <t>https://www.littelfuse.com/media?resourcetype=datasheets&amp;itemid=75e32973-b177-4ee3-a0ff-cedaf1abdb93&amp;filename=smaj-datasheet</t>
+  </si>
+  <si>
+    <t>TVS diode</t>
+  </si>
+  <si>
+    <t>C364296</t>
+  </si>
+  <si>
+    <t>Zener - 16V</t>
+  </si>
+  <si>
+    <t>C18195337</t>
+  </si>
+  <si>
+    <t>diode</t>
+  </si>
+  <si>
+    <t>C460742</t>
+  </si>
+  <si>
+    <t>thermistor</t>
+  </si>
+  <si>
+    <t>C77131</t>
+  </si>
+  <si>
+    <t>sense resistor</t>
+  </si>
+  <si>
+    <t>652-CSS2H-2512K2L30F</t>
+  </si>
+  <si>
+    <t>mouser</t>
+  </si>
+  <si>
+    <t>604k</t>
+  </si>
+  <si>
+    <t>C2484614</t>
+  </si>
+  <si>
+    <t>450k</t>
+  </si>
+  <si>
+    <t>C5159688</t>
+  </si>
+  <si>
+    <t>low rds on</t>
+  </si>
+  <si>
+    <t>vgs</t>
+  </si>
+  <si>
+    <t>Id &gt; ~15A</t>
+  </si>
+  <si>
+    <t>Vds &gt; 16.8V</t>
+  </si>
+  <si>
+    <t>nmos</t>
+  </si>
+  <si>
+    <t>C67862</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5">
+  <fonts count="11">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -165,8 +255,49 @@
       <color rgb="FF292A2E"/>
       <name val="&quot;Atlassian Sans&quot;"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FFFF0000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="10"/>
+      <color theme="10"/>
+      <name val="Arial"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF292A2E"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF333333"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -191,6 +322,18 @@
         <bgColor rgb="FFFFFFFF"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -201,10 +344,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -216,8 +360,18 @@
     <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="3">
@@ -459,22 +613,22 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:Z27"/>
+  <dimension ref="A1:Z40"/>
   <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="16.21875" customWidth="1"/>
-    <col min="2" max="2" width="16.33203125" customWidth="1"/>
+    <col min="1" max="1" width="18" customWidth="1"/>
+    <col min="2" max="2" width="18.33203125" customWidth="1"/>
     <col min="3" max="3" width="16.21875" customWidth="1"/>
-    <col min="4" max="4" width="6.6640625" customWidth="1"/>
-    <col min="5" max="5" width="15.109375" customWidth="1"/>
-    <col min="6" max="6" width="14.44140625" customWidth="1"/>
+    <col min="4" max="4" width="6.77734375" customWidth="1"/>
+    <col min="5" max="5" width="17.109375" customWidth="1"/>
+    <col min="6" max="6" width="17.88671875" customWidth="1"/>
     <col min="7" max="7" width="16" customWidth="1"/>
-    <col min="8" max="8" width="19.33203125" customWidth="1"/>
+    <col min="8" max="8" width="20.5546875" customWidth="1"/>
     <col min="9" max="9" width="17" customWidth="1"/>
-    <col min="10" max="10" width="27.33203125" customWidth="1"/>
+    <col min="10" max="10" width="37" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:26">
+    <row r="1" spans="1:26" ht="13.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -500,12 +654,31 @@
         <v>7</v>
       </c>
       <c r="I1" s="2"/>
-    </row>
-    <row r="2" spans="1:26">
+      <c r="J1" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="K1" s="7"/>
+      <c r="L1" s="7"/>
+      <c r="M1" s="7"/>
+      <c r="N1" s="7"/>
+      <c r="O1" s="7"/>
+      <c r="P1" s="7"/>
+      <c r="Q1" s="7"/>
+      <c r="R1" s="7"/>
+      <c r="S1" s="7"/>
+      <c r="T1" s="7"/>
+      <c r="U1" s="7"/>
+      <c r="V1" s="7"/>
+      <c r="W1" s="7"/>
+      <c r="X1" s="7"/>
+      <c r="Y1" s="7"/>
+      <c r="Z1" s="7"/>
+    </row>
+    <row r="2" spans="1:26" ht="13.2">
       <c r="A2" s="1"/>
       <c r="E2" s="1"/>
     </row>
-    <row r="3" spans="1:26">
+    <row r="3" spans="1:26" ht="13.2">
       <c r="A3" s="3" t="s">
         <v>8</v>
       </c>
@@ -522,10 +695,10 @@
         <v>6</v>
       </c>
       <c r="H3" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="I3" s="3" t="s">
         <v>11</v>
-      </c>
-      <c r="I3" s="3" t="s">
-        <v>12</v>
       </c>
       <c r="J3" s="1"/>
       <c r="K3" s="1"/>
@@ -545,7 +718,7 @@
       <c r="Y3" s="1"/>
       <c r="Z3" s="1"/>
     </row>
-    <row r="4" spans="1:26">
+    <row r="4" spans="1:26" ht="13.2">
       <c r="E4" s="1">
         <v>2</v>
       </c>
@@ -564,9 +737,9 @@
         <v>2.64</v>
       </c>
     </row>
-    <row r="5" spans="1:26">
+    <row r="5" spans="1:26" ht="13.2">
       <c r="A5" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B5" s="1"/>
       <c r="C5" s="1"/>
@@ -606,132 +779,319 @@
       <c r="Y5" s="1"/>
       <c r="Z5" s="1"/>
     </row>
-    <row r="6" spans="1:26">
+    <row r="6" spans="1:26" ht="13.2">
       <c r="A6" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="7" spans="1:26" ht="13.2">
+      <c r="B7" s="1" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="7" spans="1:26">
-      <c r="B7" s="1" t="s">
+      <c r="C7" s="5" t="s">
         <v>15</v>
-      </c>
-      <c r="C7" s="5" t="s">
-        <v>16</v>
       </c>
       <c r="D7" s="1">
         <v>3.3</v>
       </c>
-    </row>
-    <row r="8" spans="1:26">
+      <c r="E7">
+        <v>1</v>
+      </c>
+      <c r="H7">
+        <f>D7*G7*E7</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:26" ht="13.2">
       <c r="B8" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C8" s="6" t="s">
         <v>17</v>
-      </c>
-      <c r="C8" s="6" t="s">
-        <v>18</v>
       </c>
       <c r="D8" s="1">
         <v>3.3</v>
       </c>
+      <c r="E8">
+        <v>1</v>
+      </c>
       <c r="F8" s="1">
         <v>0.37</v>
       </c>
       <c r="G8" s="1">
         <v>0.37</v>
       </c>
+      <c r="H8">
+        <f>D8*G8*E8</f>
+        <v>1.2209999999999999</v>
+      </c>
       <c r="J8" s="1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="9" spans="1:26" ht="13.2">
+      <c r="B9" s="1" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="9" spans="1:26">
-      <c r="B9" s="1" t="s">
+      <c r="C9" s="5" t="s">
         <v>20</v>
-      </c>
-      <c r="C9" s="5" t="s">
-        <v>21</v>
       </c>
       <c r="D9" s="1">
         <v>3.3</v>
       </c>
+      <c r="E9">
+        <v>1</v>
+      </c>
       <c r="F9" s="1">
-        <v>7.4999999999999997E-2</v>
+        <v>0.08</v>
       </c>
       <c r="G9" s="1">
         <v>0.08</v>
       </c>
-    </row>
-    <row r="10" spans="1:26">
+      <c r="H9">
+        <f t="shared" ref="H9:H12" si="0">D9*G9*E9</f>
+        <v>0.26400000000000001</v>
+      </c>
+    </row>
+    <row r="10" spans="1:26" ht="13.2">
       <c r="B10" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C10" s="5" t="s">
         <v>22</v>
-      </c>
-      <c r="C10" s="5" t="s">
-        <v>23</v>
       </c>
       <c r="D10" s="1">
         <v>3.3</v>
       </c>
+      <c r="E10">
+        <v>1</v>
+      </c>
       <c r="F10" s="1">
         <v>0.01</v>
       </c>
       <c r="G10" s="1">
         <v>0.01</v>
       </c>
+      <c r="H10">
+        <f t="shared" si="0"/>
+        <v>3.3000000000000002E-2</v>
+      </c>
       <c r="J10" s="1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="11" spans="1:26" ht="13.2">
+      <c r="B11" s="1" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="11" spans="1:26">
-      <c r="B11" s="1" t="s">
+      <c r="H11">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:26" ht="15">
+      <c r="B12" s="13" t="s">
+        <v>37</v>
+      </c>
+      <c r="C12" s="14" t="s">
+        <v>38</v>
+      </c>
+      <c r="D12" s="13">
+        <v>3.3</v>
+      </c>
+      <c r="E12">
+        <v>1</v>
+      </c>
+      <c r="F12">
+        <f>13+1.3</f>
+        <v>14.3</v>
+      </c>
+      <c r="G12">
+        <f>13+1.3</f>
+        <v>14.3</v>
+      </c>
+      <c r="H12">
+        <f t="shared" si="0"/>
+        <v>47.19</v>
+      </c>
+    </row>
+    <row r="13" spans="1:26" ht="13.2">
+      <c r="A13" s="1" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="12" spans="1:26">
-      <c r="B12" s="1"/>
-    </row>
-    <row r="13" spans="1:26">
-      <c r="A13" s="1" t="s">
+    <row r="14" spans="1:26" ht="13.2">
+      <c r="A14" s="8" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="14" spans="1:26">
-      <c r="A14" s="1" t="s">
+      <c r="B14" s="9"/>
+      <c r="C14" s="9"/>
+      <c r="D14" s="9"/>
+      <c r="E14" s="9"/>
+      <c r="F14" s="8"/>
+      <c r="G14" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="H14" s="9"/>
+      <c r="I14" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="J14" s="9"/>
+      <c r="K14" s="9"/>
+      <c r="L14" s="9"/>
+      <c r="M14" s="9"/>
+      <c r="N14" s="9"/>
+      <c r="O14" s="9"/>
+      <c r="P14" s="9"/>
+      <c r="Q14" s="9"/>
+      <c r="R14" s="9"/>
+      <c r="S14" s="9"/>
+      <c r="T14" s="9"/>
+      <c r="U14" s="9"/>
+      <c r="V14" s="9"/>
+      <c r="W14" s="9"/>
+      <c r="X14" s="9"/>
+      <c r="Y14" s="9"/>
+      <c r="Z14" s="9"/>
+    </row>
+    <row r="15" spans="1:26" ht="13.2">
+      <c r="B15" s="10" t="s">
+        <v>33</v>
+      </c>
+      <c r="D15" s="1"/>
+      <c r="E15" s="1"/>
+      <c r="F15" s="12"/>
+      <c r="G15" s="13">
+        <f>((4*16*0.7) * 2)/(14.8*0.8)</f>
+        <v>7.5675675675675658</v>
+      </c>
+      <c r="I15" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="J15" s="11" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="16" spans="1:26" ht="15.75" customHeight="1">
+      <c r="J16" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" ht="15.75" customHeight="1">
+      <c r="A17" s="10" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" ht="13.2">
+      <c r="A24" s="1" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="15" spans="1:26">
-      <c r="B15" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="D15" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="E15" s="1">
-        <v>9</v>
-      </c>
-      <c r="F15" s="1">
-        <v>600</v>
-      </c>
-      <c r="G15" s="1">
-        <v>700</v>
-      </c>
-    </row>
-    <row r="24" spans="1:1">
-      <c r="A24" s="1" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="25" spans="1:1">
+    <row r="25" spans="1:6" ht="13.2">
       <c r="A25" s="1">
         <v>4</v>
       </c>
     </row>
-    <row r="26" spans="1:1">
+    <row r="26" spans="1:6" ht="13.2">
       <c r="A26" s="1" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="27" spans="1:1">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" ht="13.2">
       <c r="A27" s="1">
         <v>2.8</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" ht="15.75" customHeight="1">
+      <c r="E28" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" ht="15.75" customHeight="1">
+      <c r="E29" t="s">
+        <v>41</v>
+      </c>
+      <c r="F29" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" ht="15.75" customHeight="1">
+      <c r="E30" t="s">
+        <v>43</v>
+      </c>
+      <c r="F30" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" ht="15.75" customHeight="1">
+      <c r="E31" t="s">
+        <v>45</v>
+      </c>
+      <c r="F31" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" ht="15.75" customHeight="1">
+      <c r="E32" t="s">
+        <v>47</v>
+      </c>
+      <c r="F32" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="33" spans="5:7" ht="15.75" customHeight="1">
+      <c r="E33" t="s">
+        <v>49</v>
+      </c>
+      <c r="F33" s="15" t="s">
+        <v>50</v>
+      </c>
+      <c r="G33" s="10" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="34" spans="5:7" ht="15.75" customHeight="1">
+      <c r="E34" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="F34" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="35" spans="5:7" ht="15.75" customHeight="1">
+      <c r="E35" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="F35" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="36" spans="5:7" ht="15.75" customHeight="1">
+      <c r="E36" t="s">
+        <v>60</v>
+      </c>
+      <c r="F36" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="37" spans="5:7" ht="15.75" customHeight="1">
+      <c r="E37" s="10" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="38" spans="5:7" ht="15.75" customHeight="1">
+      <c r="E38" s="10" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="39" spans="5:7" ht="15.75" customHeight="1">
+      <c r="E39" s="10" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="40" spans="5:7" ht="15.75" customHeight="1">
+      <c r="E40" s="10" t="s">
+        <v>59</v>
       </c>
     </row>
   </sheetData>
@@ -750,6 +1110,9 @@
       <formula>LEN(TRIM(B5))=0</formula>
     </cfRule>
   </conditionalFormatting>
+  <hyperlinks>
+    <hyperlink ref="J15" r:id="rId1" xr:uid="{EE3D24E7-D4AB-4EEE-BAAC-B6359AB2B70B}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add fuel gauge schematic
</commit_message>
<xml_diff>
--- a/elec/power/Cubesat Power Budget.xlsx
+++ b/elec/power/Cubesat Power Budget.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\BMS\elec\power\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB026F42-160A-4756-A3DB-2321ADE1B7BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5976CFE-DAFE-47C5-9AC4-3D701D98236D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="66">
   <si>
     <t>Subsystem</t>
   </si>
@@ -219,6 +219,18 @@
   </si>
   <si>
     <t>C67862</t>
+  </si>
+  <si>
+    <t>C7220642</t>
+  </si>
+  <si>
+    <t>fuel gauge ic</t>
+  </si>
+  <si>
+    <t>603-PA2512FKF7T0R004</t>
+  </si>
+  <si>
+    <t>Yageo</t>
   </si>
 </sst>
 </file>
@@ -613,7 +625,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:Z40"/>
+  <dimension ref="A1:Z41"/>
   <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -1039,7 +1051,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="33" spans="5:7" ht="15.75" customHeight="1">
+    <row r="33" spans="5:10" ht="15.75" customHeight="1">
       <c r="E33" t="s">
         <v>49</v>
       </c>
@@ -1049,8 +1061,15 @@
       <c r="G33" s="10" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="34" spans="5:7" ht="15.75" customHeight="1">
+      <c r="H33" s="15"/>
+      <c r="I33" s="15" t="s">
+        <v>64</v>
+      </c>
+      <c r="J33" s="15" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="34" spans="5:10" ht="15.75" customHeight="1">
       <c r="E34" s="10" t="s">
         <v>52</v>
       </c>
@@ -1058,7 +1077,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="35" spans="5:7" ht="15.75" customHeight="1">
+    <row r="35" spans="5:10" ht="15.75" customHeight="1">
       <c r="E35" s="10" t="s">
         <v>54</v>
       </c>
@@ -1066,7 +1085,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="36" spans="5:7" ht="15.75" customHeight="1">
+    <row r="36" spans="5:10" ht="15.75" customHeight="1">
       <c r="E36" t="s">
         <v>60</v>
       </c>
@@ -1074,24 +1093,32 @@
         <v>61</v>
       </c>
     </row>
-    <row r="37" spans="5:7" ht="15.75" customHeight="1">
+    <row r="37" spans="5:10" ht="15.75" customHeight="1">
       <c r="E37" s="10" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="38" spans="5:7" ht="15.75" customHeight="1">
+    <row r="38" spans="5:10" ht="15.75" customHeight="1">
       <c r="E38" s="10" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="39" spans="5:7" ht="15.75" customHeight="1">
+    <row r="39" spans="5:10" ht="15.75" customHeight="1">
       <c r="E39" s="10" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="40" spans="5:7" ht="15.75" customHeight="1">
+    <row r="40" spans="5:10" ht="15.75" customHeight="1">
       <c r="E40" s="10" t="s">
         <v>59</v>
+      </c>
+    </row>
+    <row r="41" spans="5:10" ht="15.75" customHeight="1">
+      <c r="E41" s="10" t="s">
+        <v>63</v>
+      </c>
+      <c r="F41" t="s">
+        <v>62</v>
       </c>
     </row>
   </sheetData>

</xml_diff>